<commit_message>
Update OCR extraction, frontend table editor, and generated outputs
</commit_message>
<xml_diff>
--- a/Scan-to-Excel/Backend/outputs/output.xlsx
+++ b/Scan-to-Excel/Backend/outputs/output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Extracted Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,24 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +50,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9DDE5"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9DDE5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9DDE5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9DDE5"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,225 +441,500 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Date E 1e</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>pO</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>pO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Date collected</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Plot </t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sex</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1/9/78</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATE:</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DAY: DAI</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TUE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>WED</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>THU</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>FRI</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SUN</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL NUMBER STUDENTS PRESENT: 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>THOUGHT OF THE DAY:</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>DAILY CHECKLIST</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr"/>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DAILY CHECKLIST</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>[Put Y for Yes N for No for the points mentioned below]</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr"/>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Centre started on time: Y</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Students wore I-Cards: Y</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Volunteers wore I-Cards: Y</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Footwears placed properly: Y</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Prayer Conducted: Y</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr"/>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
+      <c r="I5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Explained the Thought: Y</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Physical Activity: Y</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Student's Attendance taken: Y</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Closing prayer conducted: Y</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Centre closed on Time: Y</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>CLASS DETAILS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Volunteer/Teacher's Name</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>In-time</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Out-time</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Class Taught</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>No of students</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Class Activity</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1/9/78</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 836</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1/9/78</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DS </t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1/20/78</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>a.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1/20/78</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1/20/78</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DS </t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>3/13/78</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>3/13/78</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3/13/78</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DS </t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Hurs h</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>2:40</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Wreading</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr"/>
+      <c r="I9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Apuava</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>228th</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Maathi</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>Wuiting! Readidg</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Jitnaj</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Gk</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Disha.</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr"/>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Maalti Basic</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr"/>
+      <c r="I12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr"/>
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="inlineStr"/>
+      <c r="I13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr"/>
+      <c r="E14" s="1" t="inlineStr"/>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="inlineStr"/>
+      <c r="I14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr"/>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr"/>
+      <c r="E15" s="1" t="inlineStr"/>
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="inlineStr"/>
+      <c r="I15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr"/>
+      <c r="E16" s="1" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr"/>
+      <c r="I16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>ANY OTHER EXTRA ACTIVITIES:</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr"/>
+      <c r="H17" s="1" t="inlineStr"/>
+      <c r="I17" s="1" t="inlineStr"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>VISITORS INFORMATION ALONG WITH CONTACT DETAILS:</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="1" t="inlineStr"/>
+      <c r="E18" s="1" t="inlineStr"/>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr"/>
+      <c r="H18" s="1" t="inlineStr"/>
+      <c r="I18" s="1" t="inlineStr"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>ANY SUGGESTION/IDEA FOR FURTHER BETTERMENT OR CHALLENGES FACED:</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr"/>
+      <c r="C19" s="1" t="inlineStr"/>
+      <c r="D19" s="1" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr"/>
+      <c r="F19" s="1" t="inlineStr"/>
+      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="inlineStr"/>
+      <c r="I19" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Improve table-first OCR extraction, add PDF support, and optimize backend performance
</commit_message>
<xml_diff>
--- a/Scan-to-Excel/Backend/outputs/output.xlsx
+++ b/Scan-to-Excel/Backend/outputs/output.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>DAY: DAI</t>
+          <t>DAY: MON</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -498,7 +498,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER STUDENTS PRESENT: 10</t>
+          <t>TOTAL NUMBER STUDENTS PRESENT:</t>
         </is>
       </c>
     </row>
@@ -508,11 +508,7 @@
           <t>THOUGHT OF THE DAY:</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>DAILY CHECKLIST</t>
-        </is>
-      </c>
+      <c r="B2" s="1" t="inlineStr"/>
       <c r="C2" s="1" t="inlineStr"/>
       <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr"/>
@@ -554,7 +550,7 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Centre started on time: Y</t>
+          <t>Centre started on time: E</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -569,12 +565,12 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Footwears placed properly: Y</t>
+          <t>Footwears placed properly:</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Prayer Conducted: Y</t>
+          <t>Prayer Conducted:</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr"/>
@@ -590,7 +586,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Physical Activity: Y</t>
+          <t>Physical Activity: 2</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -600,12 +596,12 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Closing prayer conducted: Y</t>
+          <t>Closing prayer conducted:</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Centre closed on Time: Y</t>
+          <t>Centre closed on Time:</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr"/>
@@ -702,11 +698,7 @@
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr"/>
-      <c r="G9" s="1" t="inlineStr">
-        <is>
-          <t>Wreading</t>
-        </is>
-      </c>
+      <c r="G9" s="1" t="inlineStr"/>
       <c r="H9" s="1" t="inlineStr"/>
       <c r="I9" s="1" t="inlineStr"/>
     </row>
@@ -741,16 +733,8 @@
           <t>3</t>
         </is>
       </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>Maathi</t>
-        </is>
-      </c>
-      <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>Wuiting! Readidg</t>
-        </is>
-      </c>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
       <c r="I10" s="1" t="inlineStr"/>
     </row>
     <row r="11" ht="34" customHeight="1">
@@ -784,16 +768,8 @@
           <t>2</t>
         </is>
       </c>
-      <c r="G11" s="1" t="inlineStr">
-        <is>
-          <t>Gk</t>
-        </is>
-      </c>
-      <c r="H11" s="1" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr"/>
       <c r="I11" s="1" t="inlineStr"/>
     </row>
     <row r="12" ht="34" customHeight="1">
@@ -823,11 +799,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
-        <is>
-          <t>Maalti Basic</t>
-        </is>
-      </c>
+      <c r="G12" s="1" t="inlineStr"/>
       <c r="H12" s="1" t="inlineStr"/>
       <c r="I12" s="1" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Implement robust OCR correction and JTE table extraction pipeline
</commit_message>
<xml_diff>
--- a/Scan-to-Excel/Backend/outputs/output.xlsx
+++ b/Scan-to-Excel/Backend/outputs/output.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -461,44 +461,16 @@
           <t>DATE:</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>DAY: MON</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>TUE</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>WED</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>THU</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>FRI</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SAT</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>SUN</t>
-        </is>
-      </c>
+      <c r="B1" s="1" t="inlineStr"/>
+      <c r="C1" s="1" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr"/>
+      <c r="G1" s="1" t="inlineStr"/>
+      <c r="H1" s="1" t="inlineStr"/>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER STUDENTS PRESENT: 10</t>
+          <t>TOTAL NUMBER STUDENTS PRESENT: 13</t>
         </is>
       </c>
     </row>
@@ -518,12 +490,12 @@
       <c r="I2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>DAILY CHECKLIST</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>[Put Y for Yes N for No for the points mentioned below]</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
@@ -535,13 +507,29 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>[Put Y for Yes N for No for the points mentioned below]</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr"/>
-      <c r="C4" s="1" t="inlineStr"/>
-      <c r="D4" s="1" t="inlineStr"/>
-      <c r="E4" s="1" t="inlineStr"/>
+          <t>Centre started on time: Y</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Students wore I-Cards: Y</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Volunteers wore I-Cards: Y</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Footwears placed properly: Y</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Prayer Conducted: Y</t>
+        </is>
+      </c>
       <c r="F4" s="1" t="inlineStr"/>
       <c r="G4" s="1" t="inlineStr"/>
       <c r="H4" s="1" t="inlineStr"/>
@@ -550,27 +538,27 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Centre started on time: Y</t>
+          <t>Explained the Thought: Y</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Students wore I-Cards: Y</t>
+          <t>Physical Activity: Y</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Volunteers wore I-Cards: Y</t>
+          <t>Student's Attendance taken: Y</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Footwears placed properly: Y</t>
+          <t>Closing prayer conducted: Y</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Prayer Conducted: Y</t>
+          <t>Centre closed on Time: Y</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr"/>
@@ -581,105 +569,141 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Explained the Thought: Y</t>
+          <t>SN</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Physical Activity: Y</t>
+          <t>Volunteer/Teacher's Name</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Student's Attendance taken: Y</t>
+          <t>In-time</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Closing prayer conducted: Y</t>
+          <t>Out-time</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Centre closed on Time: Y</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr"/>
-      <c r="I6" s="1" t="inlineStr"/>
+          <t>Class Taught</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>No of students</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Class Activity</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>CLASS DETAILS</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Hansh</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Bajic</t>
+        </is>
+      </c>
       <c r="I7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SN</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Volunteer/Teacher's Name</t>
+          <t>Sayali</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>In-time</t>
+          <t>6:30</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Out-time</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Class Taught</t>
+          <t>8th</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>No of students</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Subject</t>
+          <t>English</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Class Activity</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
+          <t>drammes</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>Hurs h</t>
+          <t>Tanushree</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -689,161 +713,85 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
-          <t>3rd</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr"/>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>Wreading</t>
-        </is>
-      </c>
-      <c r="H9" s="1" t="inlineStr"/>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Maths</t>
+        </is>
+      </c>
       <c r="I9" s="1" t="inlineStr"/>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>Apuava</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>228</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G10" s="1" t="inlineStr">
-        <is>
-          <t>Maathi</t>
-        </is>
-      </c>
-      <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>Wuiting! Readidg</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
       <c r="I10" s="1" t="inlineStr"/>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>Jitnaj</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="inlineStr">
-        <is>
-          <t>Gk</t>
-        </is>
-      </c>
-      <c r="H11" s="1" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr"/>
       <c r="I11" s="1" t="inlineStr"/>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>Disha.</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="1" t="inlineStr"/>
       <c r="E12" s="1" t="inlineStr"/>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G12" s="1" t="inlineStr">
-        <is>
-          <t>Maalti Basic</t>
-        </is>
-      </c>
+      <c r="F12" s="1" t="inlineStr"/>
+      <c r="G12" s="1" t="inlineStr"/>
       <c r="H12" s="1" t="inlineStr"/>
       <c r="I12" s="1" t="inlineStr"/>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr"/>
-      <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
       <c r="E13" s="1" t="inlineStr"/>
       <c r="F13" s="1" t="inlineStr"/>
       <c r="G13" s="1" t="inlineStr"/>
@@ -853,20 +801,12 @@
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr"/>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr"/>
       <c r="E14" s="1" t="inlineStr"/>
       <c r="F14" s="1" t="inlineStr"/>
       <c r="G14" s="1" t="inlineStr"/>
@@ -876,20 +816,12 @@
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>ANY OTHER EXTRA ACTIVITIES:</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr"/>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr"/>
       <c r="E15" s="1" t="inlineStr"/>
       <c r="F15" s="1" t="inlineStr"/>
       <c r="G15" s="1" t="inlineStr"/>
@@ -899,20 +831,12 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>VISITORS INFORMATION ALONG WITH CONTACT DETAILS:</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr"/>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>7:40</t>
-        </is>
-      </c>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr"/>
       <c r="E16" s="1" t="inlineStr"/>
       <c r="F16" s="1" t="inlineStr"/>
       <c r="G16" s="1" t="inlineStr"/>
@@ -922,7 +846,7 @@
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>ANY OTHER EXTRA ACTIVITIES:</t>
+          <t>ANY SUGGESTION/IDEA FOR FURTHER BETTERMENT OR CHALLENGES FACED:</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr"/>
@@ -934,36 +858,6 @@
       <c r="H17" s="1" t="inlineStr"/>
       <c r="I17" s="1" t="inlineStr"/>
     </row>
-    <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>VISITORS INFORMATION ALONG WITH CONTACT DETAILS:</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr"/>
-      <c r="C18" s="1" t="inlineStr"/>
-      <c r="D18" s="1" t="inlineStr"/>
-      <c r="E18" s="1" t="inlineStr"/>
-      <c r="F18" s="1" t="inlineStr"/>
-      <c r="G18" s="1" t="inlineStr"/>
-      <c r="H18" s="1" t="inlineStr"/>
-      <c r="I18" s="1" t="inlineStr"/>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>ANY SUGGESTION/IDEA FOR FURTHER BETTERMENT OR CHALLENGES FACED:</t>
-        </is>
-      </c>
-      <c r="B19" s="1" t="inlineStr"/>
-      <c r="C19" s="1" t="inlineStr"/>
-      <c r="D19" s="1" t="inlineStr"/>
-      <c r="E19" s="1" t="inlineStr"/>
-      <c r="F19" s="1" t="inlineStr"/>
-      <c r="G19" s="1" t="inlineStr"/>
-      <c r="H19" s="1" t="inlineStr"/>
-      <c r="I19" s="1" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
render deployment: Dockerized backend for high-performance OCR support, optimized for 512MB limit
</commit_message>
<xml_diff>
--- a/Scan-to-Excel/Backend/outputs/output.xlsx
+++ b/Scan-to-Excel/Backend/outputs/output.xlsx
@@ -458,7 +458,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DATE: 24/03/26</t>
+          <t>DATE:</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr"/>
@@ -470,7 +470,7 @@
       <c r="H1" s="1" t="inlineStr"/>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL NUMBER STUDENTS PRESENT: 26</t>
+          <t>TOTAL NUMBER STUDENTS PRESENT: 13</t>
         </is>
       </c>
     </row>
@@ -480,11 +480,7 @@
           <t>THOUGHT OF THE DAY:</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>THOUGHT OF THE DAY:</t>
-        </is>
-      </c>
+      <c r="B2" s="1" t="inlineStr"/>
       <c r="C2" s="1" t="inlineStr"/>
       <c r="D2" s="1" t="inlineStr"/>
       <c r="E2" s="1" t="inlineStr"/>
@@ -562,7 +558,7 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>Centre closed on Time:</t>
+          <t>Centre closed on Time: Y</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr"/>
@@ -625,7 +621,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>I Harsh Harsh</t>
+          <t>Hansh</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -635,27 +631,27 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>6:30</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>7th</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>8h 2 2 Engligh Ehglish Pronoun Pronoun</t>
+          <t>Bajic</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -668,7 +664,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Tanushreeinten Tansheliaten</t>
+          <t>Sayali</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -678,27 +674,27 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>6:30</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>7th</t>
+          <t>8th</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>English</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>12 12 Basi Basi Basic</t>
+          <t>drammes</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -711,7 +707,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>Tanushree</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -721,13 +717,29 @@
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr"/>
-      <c r="F9" s="1" t="inlineStr"/>
-      <c r="G9" s="1" t="inlineStr"/>
-      <c r="H9" s="1" t="inlineStr"/>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Maths</t>
+        </is>
+      </c>
       <c r="I9" s="1" t="inlineStr"/>
     </row>
     <row r="10" ht="34" customHeight="1">
@@ -736,21 +748,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr"/>
       <c r="E10" s="1" t="inlineStr"/>
       <c r="F10" s="1" t="inlineStr"/>
       <c r="G10" s="1" t="inlineStr"/>
@@ -763,21 +763,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>6:30</t>
-        </is>
-      </c>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
       <c r="E11" s="1" t="inlineStr"/>
       <c r="F11" s="1" t="inlineStr"/>
       <c r="G11" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: checkpoint current changes
</commit_message>
<xml_diff>
--- a/Scan-to-Excel/Backend/outputs/output.xlsx
+++ b/Scan-to-Excel/Backend/outputs/output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Extracted Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,24 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +50,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9DDE5"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9DDE5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9DDE5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9DDE5"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,225 +441,426 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Date E 1e</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>pO</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>pO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Date collected</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Plot </t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Species</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Sex</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1/9/78</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DATE:</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr"/>
+      <c r="C1" s="1" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr"/>
+      <c r="G1" s="1" t="inlineStr"/>
+      <c r="H1" s="1" t="inlineStr"/>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL NUMBER STUDENTS PRESENT: 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>THOUGHT OF THE DAY:</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr"/>
+      <c r="C2" s="1" t="inlineStr"/>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>[Put Y for Yes N for No for the points mentioned below]</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Centre started on time: Y</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Students wore I-Cards: Y</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Volunteers wore I-Cards: Y</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Footwears placed properly: Y</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Prayer Conducted: Y</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Explained the Thought: Y</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Physical Activity: Y</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Student's Attendance taken: Y</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Closing prayer conducted: Y</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Centre closed on Time: Y</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr"/>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
+      <c r="I5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Volunteer/Teacher's Name</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>In-time</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Out-time</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Class Taught</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>No of students</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Class Activity</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1/9/78</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 836</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1/9/78</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DS </t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>1/20/78</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>a.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1/20/78</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>1/20/78</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DS </t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>3/13/78</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>3/13/78</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>DM</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3/13/78</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DS </t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Hansh</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Bajic</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sayali</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>drammes</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Tanushree</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>6:30</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Maths</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
+      <c r="I10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr"/>
+      <c r="I11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="1" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr"/>
+      <c r="F12" s="1" t="inlineStr"/>
+      <c r="G12" s="1" t="inlineStr"/>
+      <c r="H12" s="1" t="inlineStr"/>
+      <c r="I12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr"/>
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="inlineStr"/>
+      <c r="I13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr"/>
+      <c r="E14" s="1" t="inlineStr"/>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="inlineStr"/>
+      <c r="I14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>ANY OTHER EXTRA ACTIVITIES:</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr"/>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr"/>
+      <c r="E15" s="1" t="inlineStr"/>
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="inlineStr"/>
+      <c r="I15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>VISITORS INFORMATION ALONG WITH CONTACT DETAILS:</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr"/>
+      <c r="E16" s="1" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr"/>
+      <c r="I16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>ANY SUGGESTION/IDEA FOR FURTHER BETTERMENT OR CHALLENGES FACED:</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr"/>
+      <c r="H17" s="1" t="inlineStr"/>
+      <c r="I17" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>